<commit_message>
:rocket: Identification using BVAR and IV.
I made the following changes:

1. Instead of using Local projections, I use IV-BVAR to identify the IRF to monetary policies.

2. The results are robust: We can estimate the BVAR with data from 2005 and 2008 and they show the same: when using the instrument the ShockOISL, there exists price puzzle. When using the MP strategy, the prices puzzle is reduced and we can get IRF aligned with neo Keynesian models.
</commit_message>
<xml_diff>
--- a/Datos/IPC Seasonal Adjustment.xlsx
+++ b/Datos/IPC Seasonal Adjustment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bancodelarepublica-my.sharepoint.com/personal/ojaulime_banrep_gov_co/Documents/Documents/Research/MP transmission in Colombia/Monetary-Policy-Shocks-and-Central-bank-information-in-Colombia/Datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0095047-FA3A-4828-861D-C4273CFC7B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{A0095047-FA3A-4828-861D-C4273CFC7B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{668CB9C4-1846-4080-9A17-E2F944352F1B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F2267BA6-7BA9-4F9B-BF76-4533434B6FA4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F2267BA6-7BA9-4F9B-BF76-4533434B6FA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,768 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="254">
   <si>
     <t>CPI</t>
+  </si>
+  <si>
+    <t>2005/01/31</t>
+  </si>
+  <si>
+    <t>2005/02/28</t>
+  </si>
+  <si>
+    <t>2005/03/31</t>
+  </si>
+  <si>
+    <t>2005/04/30</t>
+  </si>
+  <si>
+    <t>2005/05/31</t>
+  </si>
+  <si>
+    <t>2005/06/30</t>
+  </si>
+  <si>
+    <t>2005/07/31</t>
+  </si>
+  <si>
+    <t>2005/08/31</t>
+  </si>
+  <si>
+    <t>2005/09/30</t>
+  </si>
+  <si>
+    <t>2005/10/31</t>
+  </si>
+  <si>
+    <t>2005/11/30</t>
+  </si>
+  <si>
+    <t>2005/12/31</t>
+  </si>
+  <si>
+    <t>2006/01/31</t>
+  </si>
+  <si>
+    <t>2006/02/28</t>
+  </si>
+  <si>
+    <t>2006/03/31</t>
+  </si>
+  <si>
+    <t>2006/04/30</t>
+  </si>
+  <si>
+    <t>2006/05/31</t>
+  </si>
+  <si>
+    <t>2006/06/30</t>
+  </si>
+  <si>
+    <t>2006/07/31</t>
+  </si>
+  <si>
+    <t>2006/08/31</t>
+  </si>
+  <si>
+    <t>2006/09/30</t>
+  </si>
+  <si>
+    <t>2006/10/31</t>
+  </si>
+  <si>
+    <t>2006/11/30</t>
+  </si>
+  <si>
+    <t>2006/12/31</t>
+  </si>
+  <si>
+    <t>2007/01/31</t>
+  </si>
+  <si>
+    <t>2007/02/28</t>
+  </si>
+  <si>
+    <t>2007/03/31</t>
+  </si>
+  <si>
+    <t>2007/04/30</t>
+  </si>
+  <si>
+    <t>2007/05/31</t>
+  </si>
+  <si>
+    <t>2007/06/30</t>
+  </si>
+  <si>
+    <t>2007/07/31</t>
+  </si>
+  <si>
+    <t>2007/08/31</t>
+  </si>
+  <si>
+    <t>2007/09/30</t>
+  </si>
+  <si>
+    <t>2007/10/31</t>
+  </si>
+  <si>
+    <t>2007/11/30</t>
+  </si>
+  <si>
+    <t>2007/12/31</t>
+  </si>
+  <si>
+    <t>2008/01/31</t>
+  </si>
+  <si>
+    <t>2008/02/29</t>
+  </si>
+  <si>
+    <t>2008/03/31</t>
+  </si>
+  <si>
+    <t>2008/04/30</t>
+  </si>
+  <si>
+    <t>2008/05/31</t>
+  </si>
+  <si>
+    <t>2008/06/30</t>
+  </si>
+  <si>
+    <t>2008/07/31</t>
+  </si>
+  <si>
+    <t>2008/08/31</t>
+  </si>
+  <si>
+    <t>2008/09/30</t>
+  </si>
+  <si>
+    <t>2008/10/31</t>
+  </si>
+  <si>
+    <t>2008/11/30</t>
+  </si>
+  <si>
+    <t>2008/12/31</t>
+  </si>
+  <si>
+    <t>2009/01/31</t>
+  </si>
+  <si>
+    <t>2009/02/28</t>
+  </si>
+  <si>
+    <t>2009/03/31</t>
+  </si>
+  <si>
+    <t>2009/04/30</t>
+  </si>
+  <si>
+    <t>2009/05/31</t>
+  </si>
+  <si>
+    <t>2009/06/30</t>
+  </si>
+  <si>
+    <t>2009/07/31</t>
+  </si>
+  <si>
+    <t>2009/08/31</t>
+  </si>
+  <si>
+    <t>2009/09/30</t>
+  </si>
+  <si>
+    <t>2009/10/31</t>
+  </si>
+  <si>
+    <t>2009/11/30</t>
+  </si>
+  <si>
+    <t>2009/12/31</t>
+  </si>
+  <si>
+    <t>2010/01/31</t>
+  </si>
+  <si>
+    <t>2010/02/28</t>
+  </si>
+  <si>
+    <t>2010/03/31</t>
+  </si>
+  <si>
+    <t>2010/04/30</t>
+  </si>
+  <si>
+    <t>2010/05/31</t>
+  </si>
+  <si>
+    <t>2010/06/30</t>
+  </si>
+  <si>
+    <t>2010/07/31</t>
+  </si>
+  <si>
+    <t>2010/08/31</t>
+  </si>
+  <si>
+    <t>2010/09/30</t>
+  </si>
+  <si>
+    <t>2010/10/31</t>
+  </si>
+  <si>
+    <t>2010/11/30</t>
+  </si>
+  <si>
+    <t>2010/12/31</t>
+  </si>
+  <si>
+    <t>2011/01/31</t>
+  </si>
+  <si>
+    <t>2011/02/28</t>
+  </si>
+  <si>
+    <t>2011/03/31</t>
+  </si>
+  <si>
+    <t>2011/04/30</t>
+  </si>
+  <si>
+    <t>2011/05/31</t>
+  </si>
+  <si>
+    <t>2011/06/30</t>
+  </si>
+  <si>
+    <t>2011/07/31</t>
+  </si>
+  <si>
+    <t>2011/08/31</t>
+  </si>
+  <si>
+    <t>2011/09/30</t>
+  </si>
+  <si>
+    <t>2011/10/31</t>
+  </si>
+  <si>
+    <t>2011/11/30</t>
+  </si>
+  <si>
+    <t>2011/12/31</t>
+  </si>
+  <si>
+    <t>2012/01/31</t>
+  </si>
+  <si>
+    <t>2012/02/29</t>
+  </si>
+  <si>
+    <t>2012/03/31</t>
+  </si>
+  <si>
+    <t>2012/04/30</t>
+  </si>
+  <si>
+    <t>2012/05/31</t>
+  </si>
+  <si>
+    <t>2012/06/30</t>
+  </si>
+  <si>
+    <t>2012/07/31</t>
+  </si>
+  <si>
+    <t>2012/08/31</t>
+  </si>
+  <si>
+    <t>2012/09/30</t>
+  </si>
+  <si>
+    <t>2012/10/31</t>
+  </si>
+  <si>
+    <t>2012/11/30</t>
+  </si>
+  <si>
+    <t>2012/12/31</t>
+  </si>
+  <si>
+    <t>2013/01/31</t>
+  </si>
+  <si>
+    <t>2013/02/28</t>
+  </si>
+  <si>
+    <t>2013/03/31</t>
+  </si>
+  <si>
+    <t>2013/04/30</t>
+  </si>
+  <si>
+    <t>2013/05/31</t>
+  </si>
+  <si>
+    <t>2013/06/30</t>
+  </si>
+  <si>
+    <t>2013/07/31</t>
+  </si>
+  <si>
+    <t>2013/08/31</t>
+  </si>
+  <si>
+    <t>2013/09/30</t>
+  </si>
+  <si>
+    <t>2013/10/31</t>
+  </si>
+  <si>
+    <t>2013/11/30</t>
+  </si>
+  <si>
+    <t>2013/12/31</t>
+  </si>
+  <si>
+    <t>2014/01/31</t>
+  </si>
+  <si>
+    <t>2014/02/28</t>
+  </si>
+  <si>
+    <t>2014/03/31</t>
+  </si>
+  <si>
+    <t>2014/04/30</t>
+  </si>
+  <si>
+    <t>2014/05/31</t>
+  </si>
+  <si>
+    <t>2014/06/30</t>
+  </si>
+  <si>
+    <t>2014/07/31</t>
+  </si>
+  <si>
+    <t>2014/08/31</t>
+  </si>
+  <si>
+    <t>2014/09/30</t>
+  </si>
+  <si>
+    <t>2014/10/31</t>
+  </si>
+  <si>
+    <t>2014/11/30</t>
+  </si>
+  <si>
+    <t>2014/12/31</t>
+  </si>
+  <si>
+    <t>2015/01/31</t>
+  </si>
+  <si>
+    <t>2015/02/28</t>
+  </si>
+  <si>
+    <t>2015/03/31</t>
+  </si>
+  <si>
+    <t>2015/04/30</t>
+  </si>
+  <si>
+    <t>2015/05/31</t>
+  </si>
+  <si>
+    <t>2015/06/30</t>
+  </si>
+  <si>
+    <t>2015/07/31</t>
+  </si>
+  <si>
+    <t>2015/08/31</t>
+  </si>
+  <si>
+    <t>2015/09/30</t>
+  </si>
+  <si>
+    <t>2015/10/31</t>
+  </si>
+  <si>
+    <t>2015/11/30</t>
+  </si>
+  <si>
+    <t>2015/12/31</t>
+  </si>
+  <si>
+    <t>2016/01/31</t>
+  </si>
+  <si>
+    <t>2016/02/29</t>
+  </si>
+  <si>
+    <t>2016/03/31</t>
+  </si>
+  <si>
+    <t>2016/04/30</t>
+  </si>
+  <si>
+    <t>2016/05/31</t>
+  </si>
+  <si>
+    <t>2016/06/30</t>
+  </si>
+  <si>
+    <t>2016/07/31</t>
+  </si>
+  <si>
+    <t>2016/08/31</t>
+  </si>
+  <si>
+    <t>2016/09/30</t>
+  </si>
+  <si>
+    <t>2016/10/31</t>
+  </si>
+  <si>
+    <t>2016/11/30</t>
+  </si>
+  <si>
+    <t>2016/12/31</t>
+  </si>
+  <si>
+    <t>2017/01/31</t>
+  </si>
+  <si>
+    <t>2017/02/28</t>
+  </si>
+  <si>
+    <t>2017/03/31</t>
+  </si>
+  <si>
+    <t>2017/04/30</t>
+  </si>
+  <si>
+    <t>2017/05/31</t>
+  </si>
+  <si>
+    <t>2017/06/30</t>
+  </si>
+  <si>
+    <t>2017/07/31</t>
+  </si>
+  <si>
+    <t>2017/08/31</t>
+  </si>
+  <si>
+    <t>2017/09/30</t>
+  </si>
+  <si>
+    <t>2017/10/31</t>
+  </si>
+  <si>
+    <t>2017/11/30</t>
+  </si>
+  <si>
+    <t>2017/12/31</t>
+  </si>
+  <si>
+    <t>2018/01/31</t>
+  </si>
+  <si>
+    <t>2018/02/28</t>
+  </si>
+  <si>
+    <t>2018/03/31</t>
+  </si>
+  <si>
+    <t>2018/04/30</t>
+  </si>
+  <si>
+    <t>2018/05/31</t>
+  </si>
+  <si>
+    <t>2018/06/30</t>
+  </si>
+  <si>
+    <t>2018/07/31</t>
+  </si>
+  <si>
+    <t>2018/08/31</t>
+  </si>
+  <si>
+    <t>2018/09/30</t>
+  </si>
+  <si>
+    <t>2018/10/31</t>
+  </si>
+  <si>
+    <t>2018/11/30</t>
+  </si>
+  <si>
+    <t>2018/12/31</t>
+  </si>
+  <si>
+    <t>2019/01/31</t>
+  </si>
+  <si>
+    <t>2019/02/28</t>
+  </si>
+  <si>
+    <t>2019/03/31</t>
+  </si>
+  <si>
+    <t>2019/04/30</t>
+  </si>
+  <si>
+    <t>2019/05/31</t>
+  </si>
+  <si>
+    <t>2019/06/30</t>
+  </si>
+  <si>
+    <t>2019/07/31</t>
+  </si>
+  <si>
+    <t>2019/08/31</t>
+  </si>
+  <si>
+    <t>2019/09/30</t>
+  </si>
+  <si>
+    <t>2019/10/31</t>
+  </si>
+  <si>
+    <t>2019/11/30</t>
+  </si>
+  <si>
+    <t>2019/12/31</t>
+  </si>
+  <si>
+    <t>2020/01/31</t>
+  </si>
+  <si>
+    <t>2020/02/29</t>
+  </si>
+  <si>
+    <t>2020/03/31</t>
+  </si>
+  <si>
+    <t>2020/04/30</t>
+  </si>
+  <si>
+    <t>2020/05/31</t>
+  </si>
+  <si>
+    <t>2020/06/30</t>
+  </si>
+  <si>
+    <t>2020/07/31</t>
+  </si>
+  <si>
+    <t>2020/08/31</t>
+  </si>
+  <si>
+    <t>2020/09/30</t>
+  </si>
+  <si>
+    <t>2020/10/31</t>
+  </si>
+  <si>
+    <t>2020/11/30</t>
+  </si>
+  <si>
+    <t>2020/12/31</t>
+  </si>
+  <si>
+    <t>2021/01/31</t>
+  </si>
+  <si>
+    <t>2021/02/28</t>
+  </si>
+  <si>
+    <t>2021/03/31</t>
+  </si>
+  <si>
+    <t>2021/04/30</t>
+  </si>
+  <si>
+    <t>2021/05/31</t>
+  </si>
+  <si>
+    <t>2021/06/30</t>
+  </si>
+  <si>
+    <t>2021/07/31</t>
+  </si>
+  <si>
+    <t>2021/08/31</t>
+  </si>
+  <si>
+    <t>2021/09/30</t>
+  </si>
+  <si>
+    <t>2021/10/31</t>
+  </si>
+  <si>
+    <t>2021/11/30</t>
+  </si>
+  <si>
+    <t>2021/12/31</t>
+  </si>
+  <si>
+    <t>2022/01/31</t>
+  </si>
+  <si>
+    <t>2022/02/28</t>
+  </si>
+  <si>
+    <t>2022/03/31</t>
+  </si>
+  <si>
+    <t>2022/04/30</t>
+  </si>
+  <si>
+    <t>2022/05/31</t>
+  </si>
+  <si>
+    <t>2022/06/30</t>
+  </si>
+  <si>
+    <t>2022/07/31</t>
+  </si>
+  <si>
+    <t>2022/08/31</t>
+  </si>
+  <si>
+    <t>2022/09/30</t>
+  </si>
+  <si>
+    <t>2022/10/31</t>
+  </si>
+  <si>
+    <t>2022/11/30</t>
+  </si>
+  <si>
+    <t>2022/12/31</t>
+  </si>
+  <si>
+    <t>2023/01/31</t>
+  </si>
+  <si>
+    <t>2023/02/28</t>
+  </si>
+  <si>
+    <t>2023/03/31</t>
+  </si>
+  <si>
+    <t>2023/04/30</t>
+  </si>
+  <si>
+    <t>2023/05/31</t>
+  </si>
+  <si>
+    <t>2023/06/30</t>
+  </si>
+  <si>
+    <t>2023/07/31</t>
+  </si>
+  <si>
+    <t>2023/08/31</t>
+  </si>
+  <si>
+    <t>2023/09/30</t>
+  </si>
+  <si>
+    <t>2023/10/31</t>
+  </si>
+  <si>
+    <t>2023/11/30</t>
+  </si>
+  <si>
+    <t>2023/12/31</t>
+  </si>
+  <si>
+    <t>2024/01/31</t>
+  </si>
+  <si>
+    <t>2024/02/29</t>
+  </si>
+  <si>
+    <t>2024/03/31</t>
+  </si>
+  <si>
+    <t>2024/04/30</t>
+  </si>
+  <si>
+    <t>2024/05/31</t>
+  </si>
+  <si>
+    <t>2024/06/30</t>
+  </si>
+  <si>
+    <t>2024/07/31</t>
+  </si>
+  <si>
+    <t>2024/08/31</t>
+  </si>
+  <si>
+    <t>2024/09/30</t>
+  </si>
+  <si>
+    <t>2024/10/31</t>
+  </si>
+  <si>
+    <t>2024/11/30</t>
+  </si>
+  <si>
+    <t>2024/12/31</t>
+  </si>
+  <si>
+    <t>2025/01/31</t>
+  </si>
+  <si>
+    <t>2025/02/28</t>
+  </si>
+  <si>
+    <t>2025/03/31</t>
+  </si>
+  <si>
+    <t>2025/04/30</t>
+  </si>
+  <si>
+    <t>2025/05/31</t>
+  </si>
+  <si>
+    <t>2025/06/30</t>
+  </si>
+  <si>
+    <t>2025/07/31</t>
+  </si>
+  <si>
+    <t>2025/08/31</t>
+  </si>
+  <si>
+    <t>2025/09/30</t>
+  </si>
+  <si>
+    <t>2025/10/31</t>
+  </si>
+  <si>
+    <t>2025/11/30</t>
+  </si>
+  <si>
+    <t>2025/12/31</t>
+  </si>
+  <si>
+    <t>2026/01/31</t>
   </si>
 </sst>
 </file>
@@ -411,15 +1170,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245BFE98-BACC-4B89-A29E-535B17D118CD}">
   <dimension ref="A1:F254"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
@@ -433,8 +1192,8 @@
         <v>4.0388004560577597</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3">
@@ -456,8 +1215,8 @@
         <v>2.8007367664200089E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
@@ -479,8 +1238,8 @@
         <v>3.5641525953904463E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
@@ -502,8 +1261,8 @@
         <v>2.4174911291696688E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6">
@@ -525,8 +1284,8 @@
         <v>4.2222541998500063E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7">
@@ -548,8 +1307,8 @@
         <v>5.4802758950298625E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8">
@@ -571,8 +1330,8 @@
         <v>3.9208096602800779E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
@@ -594,8 +1353,8 @@
         <v>3.2707817319801435E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10">
@@ -617,8 +1376,8 @@
         <v>6.4866279850503972E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11">
@@ -640,8 +1399,8 @@
         <v>5.7610157367298243E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="B12">
@@ -663,8 +1422,8 @@
         <v>3.0165478879400354E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
       <c r="B13">
@@ -686,8 +1445,8 @@
         <v>1.9607037433795327E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14">
@@ -709,8 +1468,8 @@
         <v>1.2794880102502404E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15">
@@ -732,8 +1491,8 @@
         <v>-2.1249519574961795E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>15</v>
       </c>
       <c r="B16">
@@ -755,8 +1514,8 @@
         <v>3.2071490132894453E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17">
@@ -778,8 +1537,8 @@
         <v>2.4146239893800825E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18">
@@ -801,8 +1560,8 @@
         <v>3.5475035541301381E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>18</v>
       </c>
       <c r="B19">
@@ -824,8 +1583,8 @@
         <v>4.5342051056795896E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>19</v>
       </c>
       <c r="B20">
@@ -847,8 +1606,8 @@
         <v>7.059745971070619E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>20</v>
       </c>
       <c r="B21">
@@ -870,8 +1629,8 @@
         <v>6.8787794259996815E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>21</v>
       </c>
       <c r="B22">
@@ -893,8 +1652,8 @@
         <v>5.2900484325100194E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>22</v>
       </c>
       <c r="B23">
@@ -916,8 +1675,8 @@
         <v>1.9291166590704734E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>23</v>
       </c>
       <c r="B24">
@@ -939,8 +1698,8 @@
         <v>4.2137709260297029E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>24</v>
       </c>
       <c r="B25">
@@ -962,8 +1721,8 @@
         <v>3.3242099994099661E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>25</v>
       </c>
       <c r="B26">
@@ -985,8 +1744,8 @@
         <v>3.5594021060800785E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>26</v>
       </c>
       <c r="B27">
@@ -1008,8 +1767,8 @@
         <v>5.1140138009397873E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>27</v>
       </c>
       <c r="B28">
@@ -1031,8 +1790,8 @@
         <v>8.5287111267797755E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>28</v>
       </c>
       <c r="B29">
@@ -1054,8 +1813,8 @@
         <v>6.9886796454099454E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>29</v>
       </c>
       <c r="B30">
@@ -1077,8 +1836,8 @@
         <v>3.2974518336299496E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>30</v>
       </c>
       <c r="B31">
@@ -1100,8 +1859,8 @@
         <v>2.3979260168403016E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>31</v>
       </c>
       <c r="B32">
@@ -1123,8 +1882,8 @@
         <v>4.4130028980804425E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>32</v>
       </c>
       <c r="B33">
@@ -1146,8 +1905,8 @@
         <v>1.6969909829294139E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>33</v>
       </c>
       <c r="B34">
@@ -1169,8 +1928,8 @@
         <v>3.5140358518201964E-3</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>34</v>
       </c>
       <c r="B35">
@@ -1192,8 +1951,8 @@
         <v>3.2650838158199136E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>35</v>
       </c>
       <c r="B36">
@@ -1215,8 +1974,8 @@
         <v>6.6578060204198763E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
       <c r="B37">
@@ -1238,8 +1997,8 @@
         <v>5.4997659642701535E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>37</v>
       </c>
       <c r="B38">
@@ -1261,8 +2020,8 @@
         <v>6.5075478473097803E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>38</v>
       </c>
       <c r="B39">
@@ -1284,8 +2043,8 @@
         <v>8.5851107745602562E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>39</v>
       </c>
       <c r="B40">
@@ -1307,8 +2066,8 @@
         <v>5.1116303865601509E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>40</v>
       </c>
       <c r="B41">
@@ -1330,8 +2089,8 @@
         <v>5.4331974279202555E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>41</v>
       </c>
       <c r="B42">
@@ -1353,8 +2112,8 @@
         <v>9.3335001029393183E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>42</v>
       </c>
       <c r="B43">
@@ -1376,8 +2135,8 @@
         <v>9.7246010569600472E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>43</v>
       </c>
       <c r="B44">
@@ -1399,8 +2158,8 @@
         <v>7.2426274246604194E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>44</v>
       </c>
       <c r="B45">
@@ -1422,8 +2181,8 @@
         <v>4.7864196304896467E-3</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>45</v>
       </c>
       <c r="B46">
@@ -1445,8 +2204,8 @@
         <v>7.431338302001933E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>46</v>
       </c>
       <c r="B47">
@@ -1468,8 +2227,8 @@
         <v>6.4659038440204597E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>47</v>
       </c>
       <c r="B48">
@@ -1491,8 +2250,8 @@
         <v>4.5549788257899237E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>48</v>
       </c>
       <c r="B49">
@@ -1514,8 +2273,8 @@
         <v>4.8193465347896591E-3</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>49</v>
       </c>
       <c r="B50">
@@ -1537,8 +2296,8 @@
         <v>1.7868260705702355E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>50</v>
       </c>
       <c r="B51">
@@ -1560,8 +2319,8 @@
         <v>2.3492515363194855E-3</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A52">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>51</v>
       </c>
       <c r="B52">
@@ -1583,8 +2342,8 @@
         <v>2.4977929385299191E-3</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A53">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>52</v>
       </c>
       <c r="B53">
@@ -1606,8 +2365,8 @@
         <v>1.9025228961400131E-3</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>53</v>
       </c>
       <c r="B54">
@@ -1629,8 +2388,8 @@
         <v>2.7536314319043242E-4</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>54</v>
       </c>
       <c r="B55">
@@ -1652,8 +2411,8 @@
         <v>5.8160807017948457E-4</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>55</v>
       </c>
       <c r="B56">
@@ -1675,8 +2434,8 @@
         <v>1.9217991412308066E-3</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>56</v>
       </c>
       <c r="B57">
@@ -1698,8 +2457,8 @@
         <v>3.0231749543894182E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A58">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>57</v>
       </c>
       <c r="B58">
@@ -1721,8 +2480,8 @@
         <v>1.3794526455406242E-3</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>58</v>
       </c>
       <c r="B59">
@@ -1744,8 +2503,8 @@
         <v>1.5274630700092828E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>59</v>
       </c>
       <c r="B60">
@@ -1767,8 +2526,8 @@
         <v>1.1619165781100449E-3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>60</v>
       </c>
       <c r="B61">
@@ -1790,8 +2549,8 @@
         <v>9.0669396608067387E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>61</v>
       </c>
       <c r="B62">
@@ -1813,8 +2572,8 @@
         <v>2.7081260206598401E-3</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>62</v>
       </c>
       <c r="B63">
@@ -1836,8 +2595,8 @@
         <v>2.5553962902193916E-3</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>63</v>
       </c>
       <c r="B64">
@@ -1859,8 +2618,8 @@
         <v>5.5857535086989429E-4</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>64</v>
       </c>
       <c r="B65">
@@ -1882,8 +2641,8 @@
         <v>3.4346301362804255E-3</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>65</v>
       </c>
       <c r="B66">
@@ -1905,8 +2664,8 @@
         <v>1.2113394916797304E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>66</v>
       </c>
       <c r="B67">
@@ -1928,8 +2687,8 @@
         <v>2.2347537484401769E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>67</v>
       </c>
       <c r="B68">
@@ -1951,8 +2710,8 @@
         <v>1.8445589907498672E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A69">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>68</v>
       </c>
       <c r="B69">
@@ -1974,8 +2733,8 @@
         <v>3.5360720179200555E-3</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>69</v>
       </c>
       <c r="B70">
@@ -1997,8 +2756,8 @@
         <v>6.4459958450058252E-4</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A71">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>70</v>
       </c>
       <c r="B71">
@@ -2020,8 +2779,8 @@
         <v>1.8002134046497531E-3</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A72">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>71</v>
       </c>
       <c r="B72">
@@ -2043,8 +2802,8 @@
         <v>3.8050617456795166E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>72</v>
       </c>
       <c r="B73">
@@ -2066,8 +2825,8 @@
         <v>6.1895236588407343E-3</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A74">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>73</v>
       </c>
       <c r="B74">
@@ -2089,8 +2848,8 @@
         <v>4.9367991529294386E-3</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A75">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>74</v>
       </c>
       <c r="B75">
@@ -2112,8 +2871,8 @@
         <v>8.1352366062059644E-4</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A76">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>75</v>
       </c>
       <c r="B76">
@@ -2135,8 +2894,8 @@
         <v>1.1657760037397935E-3</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A77">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>76</v>
       </c>
       <c r="B77">
@@ -2158,8 +2917,8 @@
         <v>3.614978780595024E-4</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A78">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>77</v>
       </c>
       <c r="B78">
@@ -2181,8 +2940,8 @@
         <v>2.8326610909505945E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A79">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>78</v>
       </c>
       <c r="B79">
@@ -2204,8 +2963,8 @@
         <v>4.3037987516294507E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A80">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>79</v>
       </c>
       <c r="B80">
@@ -2227,8 +2986,8 @@
         <v>3.6258291657302877E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A81">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>80</v>
       </c>
       <c r="B81">
@@ -2250,8 +3009,8 @@
         <v>1.941724506870024E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A82">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>81</v>
       </c>
       <c r="B82">
@@ -2273,8 +3032,8 @@
         <v>4.6043908280495316E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A83">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>82</v>
       </c>
       <c r="B83">
@@ -2296,8 +3055,8 @@
         <v>4.3760148767999496E-3</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A84">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>83</v>
       </c>
       <c r="B84">
@@ -2319,8 +3078,8 @@
         <v>3.3122672281802323E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A85">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>84</v>
       </c>
       <c r="B85">
@@ -2342,8 +3101,8 @@
         <v>3.9477590716305855E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A86">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>85</v>
       </c>
       <c r="B86">
@@ -2365,8 +3124,8 @@
         <v>3.3508122493195458E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A87">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>86</v>
       </c>
       <c r="B87">
@@ -2388,8 +3147,8 @@
         <v>1.1161702694897357E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A88">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>87</v>
       </c>
       <c r="B88">
@@ -2411,8 +3170,8 @@
         <v>-1.3836162215952186E-4</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A89">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>88</v>
       </c>
       <c r="B89">
@@ -2434,8 +3193,8 @@
         <v>6.6413128334019689E-4</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A90">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>89</v>
       </c>
       <c r="B90">
@@ -2457,8 +3216,8 @@
         <v>3.0100814883295968E-3</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A91">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>90</v>
       </c>
       <c r="B91">
@@ -2480,8 +3239,8 @@
         <v>1.9672261217902332E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A92">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>91</v>
       </c>
       <c r="B92">
@@ -2503,8 +3262,8 @@
         <v>1.8372269017801202E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A93">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>92</v>
       </c>
       <c r="B93">
@@ -2526,8 +3285,8 @@
         <v>2.582322925369418E-3</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A94">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>93</v>
       </c>
       <c r="B94">
@@ -2549,8 +3308,8 @@
         <v>4.1618751733203396E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A95">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>94</v>
       </c>
       <c r="B95">
@@ -2572,8 +3331,8 @@
         <v>3.8385574014103696E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A96">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>95</v>
       </c>
       <c r="B96">
@@ -2595,8 +3354,8 @@
         <v>8.4914699212923495E-4</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A97">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>96</v>
       </c>
       <c r="B97">
@@ -2618,8 +3377,8 @@
         <v>7.2475240336000724E-4</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A98">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>97</v>
       </c>
       <c r="B98">
@@ -2641,8 +3400,8 @@
         <v>-8.1096776931932624E-4</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A99">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>98</v>
       </c>
       <c r="B99">
@@ -2664,8 +3423,8 @@
         <v>-4.303948722705897E-4</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A100">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>99</v>
       </c>
       <c r="B100">
@@ -2687,8 +3446,8 @@
         <v>7.199284952505991E-4</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A101">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>100</v>
       </c>
       <c r="B101">
@@ -2710,8 +3469,8 @@
         <v>1.7126269895699764E-3</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A102">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>101</v>
       </c>
       <c r="B102">
@@ -2733,8 +3492,8 @@
         <v>2.6455634530897498E-3</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A103">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>102</v>
       </c>
       <c r="B103">
@@ -2756,8 +3515,8 @@
         <v>3.5778326356297185E-3</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A104">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>103</v>
       </c>
       <c r="B104">
@@ -2779,8 +3538,8 @@
         <v>2.5318105478602249E-3</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A105">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>104</v>
       </c>
       <c r="B105">
@@ -2802,8 +3561,8 @@
         <v>2.9822094942497657E-3</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A106">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>105</v>
       </c>
       <c r="B106">
@@ -2825,8 +3584,8 @@
         <v>3.9802624327505143E-3</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A107">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>106</v>
       </c>
       <c r="B107">
@@ -2848,8 +3607,8 @@
         <v>-2.8832840271064697E-4</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A108">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>107</v>
       </c>
       <c r="B108">
@@ -2871,8 +3630,8 @@
         <v>6.5097302850425365E-5</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A109">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>108</v>
       </c>
       <c r="B109">
@@ -2894,8 +3653,8 @@
         <v>2.500427031939978E-3</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A110">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>109</v>
       </c>
       <c r="B110">
@@ -2917,8 +3676,8 @@
         <v>1.1762941533701721E-3</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A111">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
         <v>110</v>
       </c>
       <c r="B111">
@@ -2940,8 +3699,8 @@
         <v>1.2583657341194154E-3</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A112">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>111</v>
       </c>
       <c r="B112">
@@ -2963,8 +3722,8 @@
         <v>2.5636074931902897E-3</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A113">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
         <v>112</v>
       </c>
       <c r="B113">
@@ -2986,8 +3745,8 @@
         <v>3.6779221718603594E-3</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A114">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>113</v>
       </c>
       <c r="B114">
@@ -3009,8 +3768,8 @@
         <v>4.7265196255095177E-3</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A115">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>114</v>
       </c>
       <c r="B115">
@@ -3032,8 +3791,8 @@
         <v>2.5303260612901113E-3</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A116">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>115</v>
       </c>
       <c r="B116">
@@ -3055,8 +3814,8 @@
         <v>3.4973369983397617E-3</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A117">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
         <v>116</v>
       </c>
       <c r="B117">
@@ -3078,8 +3837,8 @@
         <v>4.2020415129702116E-3</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A118">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
         <v>117</v>
       </c>
       <c r="B118">
@@ -3101,8 +3860,8 @@
         <v>2.4719485088002813E-3</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A119">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
         <v>118</v>
       </c>
       <c r="B119">
@@ -3124,8 +3883,8 @@
         <v>3.8526715586497673E-3</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A120">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
         <v>119</v>
       </c>
       <c r="B120">
@@ -3147,8 +3906,8 @@
         <v>3.4435967341099882E-3</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A121">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
         <v>120</v>
       </c>
       <c r="B121">
@@ -3170,8 +3929,8 @@
         <v>2.5675177891404388E-3</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A122">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
         <v>121</v>
       </c>
       <c r="B122">
@@ -3193,8 +3952,8 @@
         <v>2.6013448378892079E-3</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A123">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>122</v>
       </c>
       <c r="B123">
@@ -3216,8 +3975,8 @@
         <v>6.3650093846607803E-3</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A124">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>123</v>
       </c>
       <c r="B124">
@@ -3239,8 +3998,8 @@
         <v>4.296858387059288E-3</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A125">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
         <v>124</v>
       </c>
       <c r="B125">
@@ -3262,8 +4021,8 @@
         <v>4.4455836445607133E-3</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A126">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>125</v>
       </c>
       <c r="B126">
@@ -3285,8 +4044,8 @@
         <v>2.7075374965193078E-3</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A127">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
         <v>126</v>
       </c>
       <c r="B127">
@@ -3308,8 +4067,8 @@
         <v>2.8321160587099214E-3</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A128">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>127</v>
       </c>
       <c r="B128">
@@ -3331,8 +4090,8 @@
         <v>3.9304408101008548E-3</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A129">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
         <v>128</v>
       </c>
       <c r="B129">
@@ -3354,8 +4113,8 @@
         <v>7.0381539181294528E-3</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A130">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>129</v>
       </c>
       <c r="B130">
@@ -3377,8 +4136,8 @@
         <v>8.2563590664301856E-3</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A131">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>130</v>
       </c>
       <c r="B131">
@@ -3400,8 +4159,8 @@
         <v>9.0180651612499219E-3</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A132">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
         <v>131</v>
       </c>
       <c r="B132">
@@ -3423,8 +4182,8 @@
         <v>8.0838153352598141E-3</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A133">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
         <v>132</v>
       </c>
       <c r="B133">
@@ -3446,8 +4205,8 @@
         <v>5.9736766912799055E-3</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A134">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
         <v>133</v>
       </c>
       <c r="B134">
@@ -3469,8 +4228,8 @@
         <v>8.9035747469203841E-3</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A135">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
         <v>134</v>
       </c>
       <c r="B135">
@@ -3492,8 +4251,8 @@
         <v>7.5326776528594763E-3</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A136">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
         <v>135</v>
       </c>
       <c r="B136">
@@ -3515,8 +4274,8 @@
         <v>7.7616047582003134E-3</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A137">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
         <v>136</v>
       </c>
       <c r="B137">
@@ -3538,8 +4297,8 @@
         <v>4.0059529634097757E-3</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A138">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
         <v>137</v>
       </c>
       <c r="B138">
@@ -3561,8 +4320,8 @@
         <v>5.27820058159989E-3</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A139">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
         <v>138</v>
       </c>
       <c r="B139">
@@ -3584,8 +4343,8 @@
         <v>6.5439761160508425E-3</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A140">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
         <v>139</v>
       </c>
       <c r="B140">
@@ -3607,8 +4366,8 @@
         <v>7.1626669151196865E-3</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A141">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
         <v>140</v>
       </c>
       <c r="B141">
@@ -3630,8 +4389,8 @@
         <v>-7.4256595920019208E-4</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A142">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>141</v>
       </c>
       <c r="B142">
@@ -3653,8 +4412,8 @@
         <v>7.88434299099805E-4</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A143">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>142</v>
       </c>
       <c r="B143">
@@ -3676,8 +4435,8 @@
         <v>1.6835379322204247E-3</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A144">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
         <v>143</v>
       </c>
       <c r="B144">
@@ -3699,8 +4458,8 @@
         <v>3.1977479109599471E-3</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A145">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
         <v>144</v>
       </c>
       <c r="B145">
@@ -3722,8 +4481,8 @@
         <v>3.8018618417297034E-3</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A146">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
         <v>145</v>
       </c>
       <c r="B146">
@@ -3745,8 +4504,8 @@
         <v>6.3100829461903984E-3</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A147">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
         <v>146</v>
       </c>
       <c r="B147">
@@ -3768,8 +4527,8 @@
         <v>4.9069097169098796E-3</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A148">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
         <v>147</v>
       </c>
       <c r="B148">
@@ -3791,8 +4550,8 @@
         <v>3.1194407101997612E-3</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A149">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
         <v>148</v>
       </c>
       <c r="B149">
@@ -3814,8 +4573,8 @@
         <v>3.6357412732703764E-3</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A150">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
         <v>149</v>
       </c>
       <c r="B150">
@@ -3837,8 +4596,8 @@
         <v>2.3029931527096537E-3</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A151">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
         <v>150</v>
       </c>
       <c r="B151">
@@ -3860,8 +4619,8 @@
         <v>3.044418187790221E-3</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A152">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
         <v>151</v>
       </c>
       <c r="B152">
@@ -3883,8 +4642,8 @@
         <v>1.4990616482295493E-3</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A153">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
         <v>152</v>
       </c>
       <c r="B153">
@@ -3906,8 +4665,8 @@
         <v>3.6332486409706988E-3</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A154">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
         <v>153</v>
       </c>
       <c r="B154">
@@ -3929,8 +4688,8 @@
         <v>1.6117099759798137E-3</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A155">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
         <v>154</v>
       </c>
       <c r="B155">
@@ -3952,8 +4711,8 @@
         <v>2.4265442469397769E-3</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A156">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
         <v>155</v>
       </c>
       <c r="B156">
@@ -3975,8 +4734,8 @@
         <v>3.8628440035601841E-3</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A157">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
         <v>156</v>
       </c>
       <c r="B157">
@@ -3998,8 +4757,8 @@
         <v>3.4638551259202899E-3</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A158">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
         <v>157</v>
       </c>
       <c r="B158">
@@ -4021,8 +4780,8 @@
         <v>2.5951023386197036E-3</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A159">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
         <v>158</v>
       </c>
       <c r="B159">
@@ -4044,8 +4803,8 @@
         <v>2.2865652914401124E-3</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A160">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>159</v>
       </c>
       <c r="B160">
@@ -4067,8 +4826,8 @@
         <v>7.4675017159009371E-4</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A161">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
         <v>160</v>
       </c>
       <c r="B161">
@@ -4090,8 +4849,8 @@
         <v>3.4740006576496896E-3</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A162">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
         <v>161</v>
       </c>
       <c r="B162">
@@ -4113,8 +4872,8 @@
         <v>2.5623275409696333E-3</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A163">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
         <v>162</v>
       </c>
       <c r="B163">
@@ -4136,8 +4895,8 @@
         <v>3.554171415740548E-3</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A164">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
         <v>163</v>
       </c>
       <c r="B164">
@@ -4159,8 +4918,8 @@
         <v>6.704282665301875E-4</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A165">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
         <v>164</v>
       </c>
       <c r="B165">
@@ -4182,8 +4941,8 @@
         <v>3.1791966930398985E-3</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A166">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
         <v>165</v>
       </c>
       <c r="B166">
@@ -4205,8 +4964,8 @@
         <v>2.6781894505294446E-3</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A167">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
         <v>166</v>
       </c>
       <c r="B167">
@@ -4228,8 +4987,8 @@
         <v>3.4735406948307457E-3</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A168">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
         <v>167</v>
       </c>
       <c r="B168">
@@ -4251,8 +5010,8 @@
         <v>3.1873476850092786E-3</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A169">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
         <v>168</v>
       </c>
       <c r="B169">
@@ -4274,8 +5033,8 @@
         <v>2.6239061957200605E-3</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A170">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
         <v>169</v>
       </c>
       <c r="B170">
@@ -4297,8 +5056,8 @@
         <v>2.6161862333005104E-3</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A171">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
         <v>170</v>
       </c>
       <c r="B171">
@@ -4320,8 +5079,8 @@
         <v>1.2181405998701322E-3</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A172">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
         <v>171</v>
       </c>
       <c r="B172">
@@ -4343,8 +5102,8 @@
         <v>2.638746783999224E-3</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A173">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
         <v>172</v>
       </c>
       <c r="B173">
@@ -4366,8 +5125,8 @@
         <v>3.6700886543403755E-3</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A174">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
         <v>173</v>
       </c>
       <c r="B174">
@@ -4389,8 +5148,8 @@
         <v>3.0986056359001424E-3</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A175">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
         <v>174</v>
       </c>
       <c r="B175">
@@ -4412,8 +5171,8 @@
         <v>4.8986247023501406E-3</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A176">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
         <v>175</v>
       </c>
       <c r="B176">
@@ -4435,8 +5194,8 @@
         <v>4.0424359949495781E-3</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A177">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
         <v>176</v>
       </c>
       <c r="B177">
@@ -4458,8 +5217,8 @@
         <v>2.6695471413704652E-3</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A178">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
         <v>177</v>
       </c>
       <c r="B178">
@@ -4481,8 +5240,8 @@
         <v>2.9633936625597102E-3</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A179">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
         <v>178</v>
       </c>
       <c r="B179">
@@ -4504,8 +5263,8 @@
         <v>3.9174321480102137E-3</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A180">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
         <v>179</v>
       </c>
       <c r="B180">
@@ -4527,8 +5286,8 @@
         <v>3.2774586248098814E-3</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A181">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
         <v>180</v>
       </c>
       <c r="B181">
@@ -4550,8 +5309,8 @@
         <v>2.0959288406299237E-3</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A182">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
         <v>181</v>
       </c>
       <c r="B182">
@@ -4573,8 +5332,8 @@
         <v>-1.3114447496205273E-3</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A183">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
         <v>182</v>
       </c>
       <c r="B183">
@@ -4596,8 +5355,8 @@
         <v>6.6928254419762467E-3</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A184">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
         <v>183</v>
       </c>
       <c r="B184">
@@ -4619,8 +5378,8 @@
         <v>5.6065144244330511E-3</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A185">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
         <v>184</v>
       </c>
       <c r="B185">
@@ -4642,8 +5401,8 @@
         <v>1.6096201931929954E-3</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A186">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
         <v>185</v>
       </c>
       <c r="B186">
@@ -4665,8 +5424,8 @@
         <v>-3.2218354411659433E-3</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A187">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
         <v>186</v>
       </c>
       <c r="B187">
@@ -4688,8 +5447,8 @@
         <v>-3.7084623873191447E-3</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A188">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
         <v>187</v>
       </c>
       <c r="B188">
@@ -4711,8 +5470,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A189">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
         <v>188</v>
       </c>
       <c r="B189">
@@ -4734,8 +5493,8 @@
         <v>-9.5269851928314608E-5</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A190">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
         <v>189</v>
       </c>
       <c r="B190">
@@ -4757,8 +5516,8 @@
         <v>3.1391226728896271E-3</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A191">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
         <v>190</v>
       </c>
       <c r="B191">
@@ -4780,8 +5539,8 @@
         <v>-5.7001711594750759E-4</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A192">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
         <v>191</v>
       </c>
       <c r="B192">
@@ -4803,8 +5562,8 @@
         <v>-1.4264659353813158E-3</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A193">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
         <v>192</v>
       </c>
       <c r="B193">
@@ -4826,8 +5585,8 @@
         <v>3.7993966677465352E-3</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A194">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
         <v>193</v>
       </c>
       <c r="B194">
@@ -4849,8 +5608,8 @@
         <v>4.0683153704916819E-3</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A195">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
         <v>194</v>
       </c>
       <c r="B195">
@@ -4872,8 +5631,8 @@
         <v>6.3062000130589269E-3</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A196">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
         <v>195</v>
       </c>
       <c r="B196">
@@ -4887,16 +5646,16 @@
         <v>4.6739497013829174</v>
       </c>
       <c r="E196">
-        <f t="shared" ref="E196:E254" si="10">C196-C195</f>
+        <f t="shared" ref="E196:E253" si="10">C196-C195</f>
         <v>3.2694262162200616E-3</v>
       </c>
       <c r="F196">
-        <f t="shared" ref="F196:F254" si="11">D196-D195</f>
+        <f t="shared" ref="F196:F253" si="11">D196-D195</f>
         <v>5.0538245142810467E-3</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A197">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
         <v>196</v>
       </c>
       <c r="B197">
@@ -4918,8 +5677,8 @@
         <v>5.9568307191915082E-3</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A198">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
         <v>197</v>
       </c>
       <c r="B198">
@@ -4941,8 +5700,8 @@
         <v>9.9723818129362485E-3</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A199">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
         <v>198</v>
       </c>
       <c r="B199">
@@ -4964,8 +5723,8 @@
         <v>-5.514199202307779E-4</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A200">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
         <v>199</v>
       </c>
       <c r="B200">
@@ -4987,8 +5746,8 @@
         <v>3.3039677632711317E-3</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A201">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
         <v>200</v>
       </c>
       <c r="B201">
@@ -5010,8 +5769,8 @@
         <v>4.3883778598852174E-3</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A202">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
         <v>201</v>
       </c>
       <c r="B202">
@@ -5033,8 +5792,8 @@
         <v>3.8240964384028686E-3</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A203">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
         <v>202</v>
       </c>
       <c r="B203">
@@ -5056,8 +5815,8 @@
         <v>1.8173557523937234E-4</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A204">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
         <v>203</v>
       </c>
       <c r="B204">
@@ -5079,8 +5838,8 @@
         <v>4.8944174566214471E-3</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A205">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
         <v>204</v>
       </c>
       <c r="B205">
@@ -5102,8 +5861,8 @@
         <v>7.2970009829909088E-3</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A206">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
         <v>205</v>
       </c>
       <c r="B206">
@@ -5125,8 +5884,8 @@
         <v>1.6468970614433864E-2</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A207">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
         <v>206</v>
       </c>
       <c r="B207">
@@ -5148,8 +5907,8 @@
         <v>1.6202132241311062E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A208">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
         <v>207</v>
       </c>
       <c r="B208">
@@ -5171,8 +5930,8 @@
         <v>9.9408693462343933E-3</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A209">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
         <v>208</v>
       </c>
       <c r="B209">
@@ -5194,8 +5953,8 @@
         <v>1.2394910151184213E-2</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A210">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
         <v>209</v>
       </c>
       <c r="B210">
@@ -5217,8 +5976,8 @@
         <v>8.3753291912334049E-3</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A211">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
         <v>210</v>
       </c>
       <c r="B211">
@@ -5240,8 +5999,8 @@
         <v>5.125846272086676E-3</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A212">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
         <v>211</v>
       </c>
       <c r="B212">
@@ -5263,8 +6022,8 @@
         <v>8.0140674348161411E-3</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A213">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
         <v>212</v>
       </c>
       <c r="B213">
@@ -5286,8 +6045,8 @@
         <v>1.0175047458077735E-2</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A214">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
         <v>213</v>
       </c>
       <c r="B214">
@@ -5309,8 +6068,8 @@
         <v>9.2574289933313736E-3</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A215">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
         <v>214</v>
       </c>
       <c r="B215">
@@ -5332,8 +6091,8 @@
         <v>7.1504326759885828E-3</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A216">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
         <v>215</v>
       </c>
       <c r="B216">
@@ -5355,8 +6114,8 @@
         <v>7.6622546911488953E-3</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A217">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
         <v>216</v>
       </c>
       <c r="B217">
@@ -5378,8 +6137,8 @@
         <v>1.2535594708328546E-2</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A218">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
         <v>217</v>
       </c>
       <c r="B218">
@@ -5401,8 +6160,8 @@
         <v>1.7617443462358828E-2</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A219">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
         <v>218</v>
       </c>
       <c r="B219">
@@ -5424,8 +6183,8 @@
         <v>1.6469232180793547E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A220">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
         <v>219</v>
       </c>
       <c r="B220">
@@ -5447,8 +6206,8 @@
         <v>1.0451329064608217E-2</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A221">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
         <v>220</v>
       </c>
       <c r="B221">
@@ -5470,8 +6229,8 @@
         <v>7.7862584851731143E-3</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A222">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
         <v>221</v>
       </c>
       <c r="B222">
@@ -5493,8 +6252,8 @@
         <v>4.3579601618262132E-3</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A223">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
         <v>222</v>
       </c>
       <c r="B223">
@@ -5516,8 +6275,8 @@
         <v>2.994462486102023E-3</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A224">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
         <v>223</v>
       </c>
       <c r="B224">
@@ -5539,8 +6298,8 @@
         <v>4.9957230246118201E-3</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A225">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
         <v>224</v>
       </c>
       <c r="B225">
@@ -5562,8 +6321,8 @@
         <v>6.9671197921454819E-3</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A226">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
         <v>225</v>
       </c>
       <c r="B226">
@@ -5585,8 +6344,8 @@
         <v>5.3038798369628992E-3</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A227">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
         <v>226</v>
       </c>
       <c r="B227">
@@ -5608,8 +6367,8 @@
         <v>2.4948648103650939E-3</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A228">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
         <v>227</v>
       </c>
       <c r="B228">
@@ -5631,8 +6390,8 @@
         <v>4.6793972934615624E-3</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A229">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
         <v>228</v>
       </c>
       <c r="B229">
@@ -5654,8 +6413,8 @@
         <v>4.5849940225135555E-3</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A230">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
         <v>229</v>
       </c>
       <c r="B230">
@@ -5677,8 +6436,8 @@
         <v>9.1073994158588079E-3</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A231">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
         <v>230</v>
       </c>
       <c r="B231">
@@ -5700,8 +6459,8 @@
         <v>1.0806273977379099E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A232">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
         <v>231</v>
       </c>
       <c r="B232">
@@ -5723,8 +6482,8 @@
         <v>7.0220524737196754E-3</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A233">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
         <v>232</v>
       </c>
       <c r="B233">
@@ -5746,8 +6505,8 @@
         <v>5.9196790202991068E-3</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A234">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
         <v>233</v>
       </c>
       <c r="B234">
@@ -5769,8 +6528,8 @@
         <v>4.2069897976295678E-3</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A235">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
         <v>234</v>
       </c>
       <c r="B235">
@@ -5792,8 +6551,8 @@
         <v>3.2134152695171281E-3</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A236">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
         <v>235</v>
       </c>
       <c r="B236">
@@ -5815,8 +6574,8 @@
         <v>2.0205545979017359E-3</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A237">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
         <v>236</v>
       </c>
       <c r="B237">
@@ -5838,8 +6597,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A238">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
         <v>237</v>
       </c>
       <c r="B238">
@@ -5861,8 +6620,8 @@
         <v>2.4331757980933233E-3</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A239">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
         <v>238</v>
       </c>
       <c r="B239">
@@ -5884,8 +6643,8 @@
         <v>-1.3201322049232189E-3</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A240">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
         <v>239</v>
       </c>
       <c r="B240">
@@ -5907,8 +6666,8 @@
         <v>2.7078648728160459E-3</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A241">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
         <v>240</v>
       </c>
       <c r="B241">
@@ -5930,8 +6689,8 @@
         <v>4.5659020865436162E-3</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A242">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
         <v>241</v>
       </c>
       <c r="B242">
@@ -5953,8 +6712,8 @@
         <v>9.3432941306827999E-3</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A243">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
         <v>242</v>
       </c>
       <c r="B243">
@@ -5976,8 +6735,8 @@
         <v>1.1287262010913679E-2</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A244">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
         <v>243</v>
       </c>
       <c r="B244">
@@ -5999,8 +6758,8 @@
         <v>5.2599757122973045E-3</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A245">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
         <v>244</v>
       </c>
       <c r="B245">
@@ -6022,8 +6781,8 @@
         <v>6.5697092231609133E-3</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A246">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
         <v>245</v>
       </c>
       <c r="B246">
@@ -6045,8 +6804,8 @@
         <v>3.2021374926438639E-3</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A247">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
         <v>246</v>
       </c>
       <c r="B247">
@@ -6068,8 +6827,8 @@
         <v>1.0651046140726095E-3</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A248">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
         <v>247</v>
       </c>
       <c r="B248">
@@ -6091,8 +6850,8 @@
         <v>2.7241636726564877E-3</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A249">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
         <v>248</v>
       </c>
       <c r="B249">
@@ -6114,8 +6873,8 @@
         <v>1.8561490247934742E-3</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A250">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
         <v>249</v>
       </c>
       <c r="B250">
@@ -6137,8 +6896,8 @@
         <v>3.2399935772158273E-3</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A251">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
         <v>250</v>
       </c>
       <c r="B251">
@@ -6160,8 +6919,8 @@
         <v>1.8467225931644293E-3</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A252">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
         <v>251</v>
       </c>
       <c r="B252">
@@ -6183,8 +6942,8 @@
         <v>7.2456611541937832E-4</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A253">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
         <v>252</v>
       </c>
       <c r="B253">
@@ -6206,8 +6965,8 @@
         <v>2.6303691104629934E-3</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A254">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
         <v>253</v>
       </c>
       <c r="B254">

</xml_diff>